<commit_message>
Add 283 test cases from screen-by-screen UIKit code audit - Total: 1,421
New coverage areas:
- Credentials Screen (region, App ID, Auth Key, SDK init)
- Login Screen (sample users, custom UID, auto-redirect, fallback)
- Home Screen (tabs, empty states, theme, mobile responsive)
- Context Menu / Logout / New Chat flows
- Create Group (public/private/password types)
- Join Password Group (dialog, validation, auto-focus)
- User Details Side Panel (block/unblock, delete chat)
- Group Details Side Panel (members, leave, transfer, delete & exit)
- Threaded Messages (thread view, search highlighting)
- Message Search / Conversations Search
- Blocked User Flow (composer, unblock link)
- Call Log Details (participants, recordings, history)
- Transfer Ownership, Banned Members, Add Members
- AI Assistant Chat, Toast Notifications, Alert Popup
- Message Delivery, Fresh Chat detection
</commit_message>
<xml_diff>
--- a/Send_Message/Send_Message_Test_Cases.xlsx
+++ b/Send_Message/Send_Message_Test_Cases.xlsx
@@ -51,7 +51,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -65,11 +65,12 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -77,6 +78,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H110"/>
+  <dimension ref="A1:H120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3519,838 +3524,1273 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n"/>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>MSG_006</t>
+        </is>
+      </c>
       <c r="B89" s="2" t="n"/>
       <c r="C89" s="2" t="n"/>
       <c r="D89" s="2" t="n"/>
-      <c r="E89" s="2" t="n"/>
-      <c r="F89" s="2" t="n"/>
-      <c r="G89" s="2" t="n"/>
-      <c r="H89" s="2" t="n"/>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>Verify message with only spaces</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>1. Open any chat conversation.
+2. Type only spaces.
+3. Click send button.</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>Message should not be sent; spaces-only input should be treated as empty.</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
+          <t>MSG_019</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n"/>
+      <c r="C90" s="2" t="n"/>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and chat is open</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Verify extremely long message handling</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>1. Type a 10000+ character message.
+2. Click send.</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Application should handle gracefully; either send or show character limit warning.</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Low / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>MSG_045</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="n"/>
+      <c r="C91" s="2" t="n"/>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in, network error</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Verify message retry on failure</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>1. Send message during network error.
+2. Observe failed message.
+3. Click retry.</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>Retry option should be available; message should resend on retry.</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>MSG_053</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n"/>
+      <c r="C92" s="2" t="n"/>
+      <c r="D92" s="2" t="n"/>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Verify file size limit handling</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>1. Click attachment icon.
+2. Select file exceeding size limit.</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Error message should display indicating file size limit exceeded.</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>High / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>MSG_054</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="n"/>
+      <c r="C93" s="2" t="n"/>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in, network error</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>Verify attachment upload failure handling</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>1. Disconnect network.
+2. Try to send attachment.</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>Error message should display; retry option should be available.</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>MSG_062</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and chat is open</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Verify very short recording handling</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>1. Press and release recording button quickly (&lt; 1 second).</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>Recording should be cancelled or warning should display.</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Low / Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>MSG_093</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="n"/>
+      <c r="C95" s="2" t="n"/>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and one-on-one chat is open</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>Verify @ mention in direct chat</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>1. Open one-on-one chat.
+2. Type "@".</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>Only the other user should appear in suggestions (or feature disabled).</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>Low / Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>MSG_107</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n"/>
+      <c r="C96" s="2" t="n"/>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in, network disconnected</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>Verify audio message fails without network</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>1. Disconnect network.
+2. Try to send an audio message.</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>Error message should display or upload should queue with retry option.</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>MSG_108</t>
+        </is>
+      </c>
+      <c r="B97" s="2" t="n"/>
+      <c r="C97" s="2" t="n"/>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and chat is open</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>Verify unsupported audio format</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>1. Try to send an unsupported audio file format.</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>Error message should display or file should be rejected.</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>MSG_143</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Blocked User - Composer Hidden</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>User is blocked</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>Verify composer replaced with blocked message</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>1. Open conversation with blocked user
+2. Observe composer area</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>Composer should be hidden, 'Cannot send to blocked user' message displayed</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>MSG_144</t>
+        </is>
+      </c>
+      <c r="B99" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C99" s="2" t="inlineStr">
+        <is>
+          <t>Blocked User - Unblock From Composer</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>Blocked user message shown</t>
+        </is>
+      </c>
+      <c r="E99" s="2" t="inlineStr">
+        <is>
+          <t>Verify unblock link in composer area</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>1. Open blocked user conversation
+2. Click 'Click to unblock' link</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>User should be unblocked, composer should reappear</t>
+        </is>
+      </c>
+      <c r="H99" s="2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>MSG_145</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>Blocked User - Real-time Block Update</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>Conversation open, user blocked from details</t>
+        </is>
+      </c>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Verify composer updates when user blocked</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>1. Open conversation
+2. Block user from details panel
+3. Observe composer</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>Composer should immediately hide and show blocked message</t>
+        </is>
+      </c>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>MSG_146</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C101" s="2" t="inlineStr">
+        <is>
+          <t>Blocked User - Real-time Unblock Update</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>Blocked user conversation open</t>
+        </is>
+      </c>
+      <c r="E101" s="2" t="inlineStr">
+        <is>
+          <t>Verify composer updates when user unblocked</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>1. Open blocked user conversation
+2. Unblock from details
+3. Observe composer</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>Composer should immediately reappear</t>
+        </is>
+      </c>
+      <c r="H101" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>MSG_147</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>Delivery - Auto Mark Delivered</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>Message received while not in chat tab</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>Verify messages auto-marked as delivered</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>1. Be on Users/Groups tab
+2. Receive a message
+3. Check delivery status</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>Message should be auto-marked as delivered via CometChat.markAsDelivered()</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>MSG_148</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C103" s="2" t="inlineStr">
+        <is>
+          <t>Delivery - Skip Own Messages</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>Own message received via listener</t>
+        </is>
+      </c>
+      <c r="E103" s="2" t="inlineStr">
+        <is>
+          <t>Verify own messages not marked as delivered</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>1. Send a message
+2. Observe delivery marking</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>Messages from logged-in user should not be marked as delivered again</t>
+        </is>
+      </c>
+      <c r="H103" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>MSG_149</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C104" s="2" t="inlineStr">
+        <is>
+          <t>Delivery - Skip Already Delivered</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>Message already has deliveredAt</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>Verify already-delivered messages skipped</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>1. Receive message with deliveredAt set
+2. Observe</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>Should not call markAsDelivered for already-delivered messages</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>MSG_150</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C105" s="2" t="inlineStr">
+        <is>
+          <t>Fresh Chat - Detection</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>New chat with no messages</t>
+        </is>
+      </c>
+      <c r="E105" s="2" t="inlineStr">
+        <is>
+          <t>Verify fresh chat is detected</t>
+        </is>
+      </c>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>1. Start new conversation with user
+2. Observe state</t>
+        </is>
+      </c>
+      <c r="G105" s="2" t="inlineStr">
+        <is>
+          <t>isFreshChat should be set to true via ccActiveChatChanged event</t>
+        </is>
+      </c>
+      <c r="H105" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>MSG_151</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Fresh Chat - First Message Converts</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>Fresh chat, first message sent</t>
+        </is>
+      </c>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Verify fresh chat converts to conversation on first message</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>1. Open fresh chat
+2. Send first message
+3. Observe</t>
+        </is>
+      </c>
+      <c r="G106" s="2" t="inlineStr">
+        <is>
+          <t>isFreshChat should become false, conversation should be fetched via getConversation()</t>
+        </is>
+      </c>
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>MSG_152</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Fresh Chat - First Message Received</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>Fresh chat, message received</t>
+        </is>
+      </c>
+      <c r="E107" s="2" t="inlineStr">
+        <is>
+          <t>Verify incoming message converts fresh chat</t>
+        </is>
+      </c>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>1. Open fresh chat
+2. Receive message from other user
+3. Observe</t>
+        </is>
+      </c>
+      <c r="G107" s="2" t="inlineStr">
+        <is>
+          <t>isFreshChat should become false, conversation created</t>
+        </is>
+      </c>
+      <c r="H107" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="n"/>
+      <c r="B108" s="3" t="n"/>
+      <c r="C108" s="3" t="n"/>
+      <c r="D108" s="3" t="n"/>
+      <c r="E108" s="3" t="n"/>
+      <c r="F108" s="3" t="n"/>
+      <c r="G108" s="3" t="n"/>
+      <c r="H108" s="3" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
           <t>MSG_005</t>
         </is>
       </c>
-      <c r="B90" s="2" t="inlineStr">
+      <c r="B109" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C109" s="2" t="inlineStr">
         <is>
           <t>Verify Message Input field</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D109" s="2" t="inlineStr">
         <is>
           <t>User is logged in and chat is open</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr">
+      <c r="E109" s="2" t="inlineStr">
         <is>
           <t>Verify empty message cannot be sent</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr">
+      <c r="F109" s="2" t="inlineStr">
         <is>
           <t>1. Open any chat conversation.
 2. Leave input field empty.
 3. Click send button.</t>
         </is>
       </c>
-      <c r="G90" s="2" t="inlineStr">
+      <c r="G109" s="2" t="inlineStr">
         <is>
           <t>Send button should be disabled or message should not be sent.</t>
         </is>
       </c>
-      <c r="H90" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>MSG_006</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>Verify message with only spaces</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>1. Open any chat conversation.
-2. Type only spaces.
-3. Click send button.</t>
-        </is>
-      </c>
-      <c r="G91" s="2" t="inlineStr">
-        <is>
-          <t>Message should not be sent; spaces-only input should be treated as empty.</t>
-        </is>
-      </c>
-      <c r="H91" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="inlineStr">
+      <c r="H109" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>MSG_011</t>
         </is>
       </c>
-      <c r="B92" s="2" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C92" s="2" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>Verify Send button</t>
         </is>
       </c>
-      <c r="D92" s="2" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>User is logged in and chat is open</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
+      <c r="E110" s="2" t="inlineStr">
         <is>
           <t>Verify send button disabled when empty</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>1. Open any chat conversation.
 2. Leave input field empty.
 3. Observe send button.</t>
         </is>
       </c>
-      <c r="G92" s="2" t="inlineStr">
+      <c r="G110" s="2" t="inlineStr">
         <is>
           <t>Send button should be disabled or grayed out.</t>
         </is>
       </c>
-      <c r="H92" s="2" t="inlineStr">
+      <c r="H110" s="2" t="inlineStr">
         <is>
           <t>High / Medium</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
         <is>
           <t>MSG_018</t>
         </is>
       </c>
-      <c r="B93" s="2" t="inlineStr">
+      <c r="B111" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
+      <c r="C111" s="2" t="inlineStr">
         <is>
           <t>Verify Text message sending</t>
         </is>
       </c>
-      <c r="D93" s="2" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>User is logged in, network disconnected</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
+      <c r="E111" s="2" t="inlineStr">
         <is>
           <t>Verify message sending fails without network</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="F111" s="2" t="inlineStr">
         <is>
           <t>1. Disconnect network.
 2. Type a message.
 3. Click send.</t>
         </is>
       </c>
-      <c r="G93" s="2" t="inlineStr">
+      <c r="G111" s="2" t="inlineStr">
         <is>
           <t>Error indicator should show; message should be queued or show failed status.</t>
         </is>
       </c>
-      <c r="H93" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>MSG_019</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="n"/>
-      <c r="C94" s="2" t="n"/>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and chat is open</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>Verify extremely long message handling</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>1. Type a 10000+ character message.
-2. Click send.</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>Application should handle gracefully; either send or show character limit warning.</t>
-        </is>
-      </c>
-      <c r="H94" s="2" t="inlineStr">
-        <is>
-          <t>Low / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="inlineStr">
+      <c r="H111" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
         <is>
           <t>MSG_030</t>
         </is>
       </c>
-      <c r="B95" s="2" t="inlineStr">
+      <c r="B112" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C95" s="2" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>Verify Enter key to send</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
         <is>
           <t>User is logged in and input is empty</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr">
+      <c r="E112" s="2" t="inlineStr">
         <is>
           <t>Verify Enter key with empty input</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>1. Leave input field empty.
 2. Press Enter key.</t>
         </is>
       </c>
-      <c r="G95" s="2" t="inlineStr">
+      <c r="G112" s="2" t="inlineStr">
         <is>
           <t>Nothing should happen; empty message should not be sent.</t>
         </is>
       </c>
-      <c r="H95" s="2" t="inlineStr">
+      <c r="H112" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="2" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
         <is>
           <t>MSG_044</t>
         </is>
       </c>
-      <c r="B96" s="2" t="inlineStr">
+      <c r="B113" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C113" s="2" t="inlineStr">
         <is>
           <t>Verify Message loading</t>
         </is>
       </c>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="D113" s="2" t="inlineStr">
         <is>
           <t>User is logged in, slow network</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr">
+      <c r="E113" s="2" t="inlineStr">
         <is>
           <t>Verify message sending with slow network</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="F113" s="2" t="inlineStr">
         <is>
           <t>1. Simulate slow network.
 2. Send a message.
 3. Observe behavior.</t>
         </is>
       </c>
-      <c r="G96" s="2" t="inlineStr">
+      <c r="G113" s="2" t="inlineStr">
         <is>
           <t>Loading indicator should show; message should eventually send or show retry option.</t>
         </is>
       </c>
-      <c r="H96" s="2" t="inlineStr">
+      <c r="H113" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>MSG_045</t>
-        </is>
-      </c>
-      <c r="B97" s="2" t="n"/>
-      <c r="C97" s="2" t="n"/>
-      <c r="D97" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in, network error</t>
-        </is>
-      </c>
-      <c r="E97" s="2" t="inlineStr">
-        <is>
-          <t>Verify message retry on failure</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr">
-        <is>
-          <t>1. Send message during network error.
-2. Observe failed message.
-3. Click retry.</t>
-        </is>
-      </c>
-      <c r="G97" s="2" t="inlineStr">
-        <is>
-          <t>Retry option should be available; message should resend on retry.</t>
-        </is>
-      </c>
-      <c r="H97" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
         <is>
           <t>MSG_052</t>
         </is>
       </c>
-      <c r="B98" s="2" t="inlineStr">
+      <c r="B114" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C114" s="2" t="inlineStr">
         <is>
           <t>Verify Attachment feature</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D114" s="2" t="inlineStr">
         <is>
           <t>User is logged in and chat is open</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E114" s="2" t="inlineStr">
         <is>
           <t>Verify unsupported file type handling</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F114" s="2" t="inlineStr">
         <is>
           <t>1. Click attachment icon.
 2. Try to select unsupported file type.</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
+      <c r="G114" s="2" t="inlineStr">
         <is>
           <t>Error message should display or file should not be selectable.</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
+      <c r="H114" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
-        <is>
-          <t>MSG_053</t>
-        </is>
-      </c>
-      <c r="B99" s="2" t="n"/>
-      <c r="C99" s="2" t="n"/>
-      <c r="D99" s="2" t="n"/>
-      <c r="E99" s="2" t="inlineStr">
-        <is>
-          <t>Verify file size limit handling</t>
-        </is>
-      </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>1. Click attachment icon.
-2. Select file exceeding size limit.</t>
-        </is>
-      </c>
-      <c r="G99" s="2" t="inlineStr">
-        <is>
-          <t>Error message should display indicating file size limit exceeded.</t>
-        </is>
-      </c>
-      <c r="H99" s="2" t="inlineStr">
-        <is>
-          <t>High / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>MSG_054</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="n"/>
-      <c r="C100" s="2" t="n"/>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in, network error</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Verify attachment upload failure handling</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>1. Disconnect network.
-2. Try to send attachment.</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr">
-        <is>
-          <t>Error message should display; retry option should be available.</t>
-        </is>
-      </c>
-      <c r="H100" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
         <is>
           <t>MSG_061</t>
         </is>
       </c>
-      <c r="B101" s="2" t="inlineStr">
+      <c r="B115" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
+      <c r="C115" s="2" t="inlineStr">
         <is>
           <t>Verify Voice Recording feature</t>
         </is>
       </c>
-      <c r="D101" s="2" t="inlineStr">
+      <c r="D115" s="2" t="inlineStr">
         <is>
           <t>User is logged in, microphone permission denied</t>
         </is>
       </c>
-      <c r="E101" s="2" t="inlineStr">
+      <c r="E115" s="2" t="inlineStr">
         <is>
           <t>Verify recording without microphone permission</t>
         </is>
       </c>
-      <c r="F101" s="2" t="inlineStr">
+      <c r="F115" s="2" t="inlineStr">
         <is>
           <t>1. Deny microphone permission.
 2. Try to record voice message.</t>
         </is>
       </c>
-      <c r="G101" s="2" t="inlineStr">
+      <c r="G115" s="2" t="inlineStr">
         <is>
           <t>Permission request should appear or error message should display.</t>
         </is>
       </c>
-      <c r="H101" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>MSG_062</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="n"/>
-      <c r="C102" s="2" t="n"/>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and chat is open</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="inlineStr">
-        <is>
-          <t>Verify very short recording handling</t>
-        </is>
-      </c>
-      <c r="F102" s="2" t="inlineStr">
-        <is>
-          <t>1. Press and release recording button quickly (&lt; 1 second).</t>
-        </is>
-      </c>
-      <c r="G102" s="2" t="inlineStr">
-        <is>
-          <t>Recording should be cancelled or warning should display.</t>
-        </is>
-      </c>
-      <c r="H102" s="2" t="inlineStr">
-        <is>
-          <t>Low / Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="2" t="inlineStr">
+      <c r="H115" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
         <is>
           <t>MSG_077</t>
         </is>
       </c>
-      <c r="B103" s="2" t="inlineStr">
+      <c r="B116" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C103" s="2" t="inlineStr">
+      <c r="C116" s="2" t="inlineStr">
         <is>
           <t>Verify Sticker feature</t>
         </is>
       </c>
-      <c r="D103" s="2" t="inlineStr">
+      <c r="D116" s="2" t="inlineStr">
         <is>
           <t>User is logged in, no sticker packs available</t>
         </is>
       </c>
-      <c r="E103" s="2" t="inlineStr">
+      <c r="E116" s="2" t="inlineStr">
         <is>
           <t>Verify empty sticker state</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr">
+      <c r="F116" s="2" t="inlineStr">
         <is>
           <t>1. Open sticker picker with no packs.
 2. Observe display.</t>
         </is>
       </c>
-      <c r="G103" s="2" t="inlineStr">
+      <c r="G116" s="2" t="inlineStr">
         <is>
           <t>Empty state or option to download sticker packs should display.</t>
         </is>
       </c>
-      <c r="H103" s="2" t="inlineStr">
+      <c r="H116" s="2" t="inlineStr">
         <is>
           <t>Low / Low</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>MSG_083</t>
         </is>
       </c>
-      <c r="B104" s="2" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C104" s="2" t="inlineStr">
+      <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Verify @all mention feature</t>
         </is>
       </c>
-      <c r="D104" s="2" t="inlineStr">
+      <c r="D117" s="2" t="inlineStr">
         <is>
           <t>User is logged in and one-on-one chat is open</t>
         </is>
       </c>
-      <c r="E104" s="2" t="inlineStr">
+      <c r="E117" s="2" t="inlineStr">
         <is>
           <t>Verify @all not available in direct chat</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr">
+      <c r="F117" s="2" t="inlineStr">
         <is>
           <t>1. Open one-on-one chat.
 2. Type "@all".</t>
         </is>
       </c>
-      <c r="G104" s="2" t="inlineStr">
+      <c r="G117" s="2" t="inlineStr">
         <is>
           <t>@all suggestion should not appear in direct/one-on-one chats.</t>
         </is>
       </c>
-      <c r="H104" s="2" t="inlineStr">
+      <c r="H117" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>MSG_092</t>
         </is>
       </c>
-      <c r="B105" s="2" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C105" s="2" t="inlineStr">
+      <c r="C118" s="2" t="inlineStr">
         <is>
           <t>Verify @ mention feature</t>
         </is>
       </c>
-      <c r="D105" s="2" t="inlineStr">
+      <c r="D118" s="2" t="inlineStr">
         <is>
           <t>User is logged in and group chat is open</t>
         </is>
       </c>
-      <c r="E105" s="2" t="inlineStr">
+      <c r="E118" s="2" t="inlineStr">
         <is>
           <t>Verify @ with no matching members</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr">
+      <c r="F118" s="2" t="inlineStr">
         <is>
           <t>1. Type "@xyz123" in input field.
 2. Observe suggestions.</t>
         </is>
       </c>
-      <c r="G105" s="2" t="inlineStr">
+      <c r="G118" s="2" t="inlineStr">
         <is>
           <t>No suggestions should appear or "No members found" message.</t>
         </is>
       </c>
-      <c r="H105" s="2" t="inlineStr">
+      <c r="H118" s="2" t="inlineStr">
         <is>
           <t>Medium / Medium</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>MSG_093</t>
-        </is>
-      </c>
-      <c r="B106" s="2" t="n"/>
-      <c r="C106" s="2" t="n"/>
-      <c r="D106" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and one-on-one chat is open</t>
-        </is>
-      </c>
-      <c r="E106" s="2" t="inlineStr">
-        <is>
-          <t>Verify @ mention in direct chat</t>
-        </is>
-      </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>1. Open one-on-one chat.
-2. Type "@".</t>
-        </is>
-      </c>
-      <c r="G106" s="2" t="inlineStr">
-        <is>
-          <t>Only the other user should appear in suggestions (or feature disabled).</t>
-        </is>
-      </c>
-      <c r="H106" s="2" t="inlineStr">
-        <is>
-          <t>Low / Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
         <is>
           <t>MSG_099</t>
         </is>
       </c>
-      <c r="B107" s="2" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="C119" s="2" t="inlineStr">
         <is>
           <t>Verify Custom Message</t>
         </is>
       </c>
-      <c r="D107" s="2" t="inlineStr">
+      <c r="D119" s="2" t="inlineStr">
         <is>
           <t>User is logged in, network disconnected</t>
         </is>
       </c>
-      <c r="E107" s="2" t="inlineStr">
+      <c r="E119" s="2" t="inlineStr">
         <is>
           <t>Verify custom message fails without network</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr">
+      <c r="F119" s="2" t="inlineStr">
         <is>
           <t>1. Disconnect network.
 2. Try to send a custom message.</t>
         </is>
       </c>
-      <c r="G107" s="2" t="inlineStr">
+      <c r="G119" s="2" t="inlineStr">
         <is>
           <t>Error message should display or message should queue with retry option.</t>
         </is>
       </c>
-      <c r="H107" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="2" t="inlineStr">
+      <c r="H119" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>MSG_106</t>
         </is>
       </c>
-      <c r="B108" s="2" t="inlineStr">
+      <c r="B120" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
         <is>
           <t>Verify Audio Message</t>
         </is>
       </c>
-      <c r="D108" s="2" t="inlineStr">
+      <c r="D120" s="2" t="inlineStr">
         <is>
           <t>User is logged in and chat is open</t>
         </is>
       </c>
-      <c r="E108" s="2" t="inlineStr">
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>Verify large audio file exceeding size limit</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr">
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>1. Try to send an audio file exceeding the size limit.</t>
         </is>
       </c>
-      <c r="G108" s="2" t="inlineStr">
+      <c r="G120" s="2" t="inlineStr">
         <is>
           <t>Error message should display indicating file size limit exceeded.</t>
         </is>
       </c>
-      <c r="H108" s="2" t="inlineStr">
+      <c r="H120" s="2" t="inlineStr">
         <is>
           <t>High / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>MSG_107</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="n"/>
-      <c r="C109" s="2" t="n"/>
-      <c r="D109" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in, network disconnected</t>
-        </is>
-      </c>
-      <c r="E109" s="2" t="inlineStr">
-        <is>
-          <t>Verify audio message fails without network</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>1. Disconnect network.
-2. Try to send an audio message.</t>
-        </is>
-      </c>
-      <c r="G109" s="2" t="inlineStr">
-        <is>
-          <t>Error message should display or upload should queue with retry option.</t>
-        </is>
-      </c>
-      <c r="H109" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>MSG_108</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="n"/>
-      <c r="C110" s="2" t="n"/>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and chat is open</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="inlineStr">
-        <is>
-          <t>Verify unsupported audio format</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>1. Try to send an unsupported audio file format.</t>
-        </is>
-      </c>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>Error message should display or file should be rejected.</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4533,6 +4973,136 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>MSG_153</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Blocked User - Event Subscription</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Conversation open</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Verify block/unblock event subscriptions</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1. Open conversation
+2. Block user
+3. Unblock user</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>ccUserBlocked and ccUserUnblocked events should update composer state</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>MSG_154</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Delivery - All Message Types</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Various message types received</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Verify delivery marking for all types</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1. Receive text, media, and custom messages
+2. Check delivery</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>All three message types should trigger markAsDelivered via respective listeners</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>MSG_155</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Fresh Chat - All Message Types Convert</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Fresh chat</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Verify all message types convert fresh chat</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>1. Send text/media/custom message in fresh chat
+2. Observe</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>ccMessageSent, onTextMessageReceived, onMediaMessageReceived, onCustomMessageReceived all handle conversion</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4542,179 +5112,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00FFC000"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TestCase_ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Sentiment</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Precondition</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Results</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Priority / Severity</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>MSG_112</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Regression: Send Message</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in and chat is open</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Verify message sending works after failed attempt</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>1. Send a message during network error (fails).
-2. Restore network.
-3. Retry sending.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Message should send successfully on retry. No duplicate messages.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>MSG_113</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Verify message order preserved after rapid sending</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>1. Send 10 messages rapidly one after another.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>All 10 messages should appear in the exact order they were sent.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>MSG_114</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Verify media message sending after app crash recovery</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>1. Start uploading a large file.
-2. Force close app.
-3. Reopen.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Upload should either resume or show failed state with retry option.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Medium / High</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00FF0000"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -4776,17 +5173,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MSG_115</t>
+          <t>MSG_112</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Security: Send Message</t>
+          <t>Regression: Send Message</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -4796,29 +5193,31 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Verify message cannot be sent to unauthorized conversation</t>
+          <t>Verify message sending works after failed attempt</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1. Try to send a message to a group you've been removed from.</t>
+          <t>1. Send a message during network error (fails).
+2. Restore network.
+3. Retry sending.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Message should fail with appropriate error. No message delivered.</t>
+          <t>Message should send successfully on retry. No duplicate messages.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>High / Critical</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MSG_116</t>
+          <t>MSG_113</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -4826,29 +5225,29 @@
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Verify file upload scans for malware (if applicable)</t>
+          <t>Verify message order preserved after rapid sending</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1. Upload a file flagged as potentially malicious.</t>
+          <t>1. Send 10 messages rapidly one after another.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>File should be rejected or quarantined based on security policy.</t>
+          <t>All 10 messages should appear in the exact order they were sent.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>High / Critical</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MSG_117</t>
+          <t>MSG_114</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -4856,18 +5255,187 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
+          <t>Verify media message sending after app crash recovery</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1. Start uploading a large file.
+2. Force close app.
+3. Reopen.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Upload should either resume or show failed state with retry option.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Medium / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n"/>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00FF0000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>MSG_116</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Verify file upload scans for malware (if applicable)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1. Upload a file flagged as potentially malicious.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>File should be rejected or quarantined based on security policy.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>High / Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>MSG_117</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Verify message encryption in transit</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>1. Send a message.
 2. Inspect network traffic.</t>
         </is>
       </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Message content should be encrypted (HTTPS/WSS). Not visible in plain text.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>High / Critical</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>MSG_118</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Verify spoofed sender ID prevention</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1. Try to send a message with a manipulated sender ID via API.</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Message content should be encrypted (HTTPS/WSS). Not visible in plain text.</t>
+          <t>Server should reject the message. Sender ID should be validated server-side.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -4877,30 +5445,52 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>MSG_118</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Verify spoofed sender ID prevention</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>1. Try to send a message with a manipulated sender ID via API.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Server should reject the message. Sender ID should be validated server-side.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>MSG_115</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Security: Send Message</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and chat is open</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Verify message cannot be sent to unauthorized conversation</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1. Try to send a message to a group you've been removed from.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Message should fail with appropriate error. No message delivered.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>High / Critical</t>
         </is>
@@ -4915,6 +5505,298 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00ED7D31"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>TestCase_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Test Scenario</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Test Case</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Results</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Priority / Severity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>MSG_119</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Edge Case: Send Message</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>User is logged in and chat is open</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Verify sending message while receiver is typing</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>1. Both users type simultaneously.
+2. Both send at the same time.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Both messages should appear in correct order. No message loss.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>MSG_120</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n"/>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Verify sending message to a user who blocked you</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1. Send a message to a user who has blocked you.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Message should fail or appear sent but not delivered. Appropriate handling per app policy.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>MSG_121</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Verify sending message immediately after joining a group</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>1. Join a new group.
+2. Immediately send a message.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Message should send successfully. Should appear for all group members.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Medium / Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>MSG_122</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n"/>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Verify sending multiple media types in sequence</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>1. Send an image.
+2. Immediately send a video.
+3. Send a document.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>All three should upload and appear in correct order. No upload conflicts.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>High / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>MSG_124</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Verify sending corrupted media file</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>1. Rename a .txt file to .jpg.
+2. Try to send as image.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>App should detect invalid file and show error. Should not crash.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Medium / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n"/>
+      <c r="B7" s="3" t="n"/>
+      <c r="C7" s="3" t="n"/>
+      <c r="D7" s="3" t="n"/>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="n"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>MSG_123</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Edge Case: Send Message</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Verify sending message with zero-width characters</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>1. Send a message containing only zero-width unicode characters.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Message should be blocked or displayed as empty. No invisible messages.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Medium / High</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
+      <c r="C9" s="4" t="n"/>
+      <c r="D9" s="4" t="n"/>
+      <c r="E9" s="4" t="n"/>
+      <c r="F9" s="4" t="n"/>
+      <c r="G9" s="4" t="n"/>
+      <c r="H9" s="4" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -4976,7 +5858,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MSG_119</t>
+          <t>MSG_125</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -4986,7 +5868,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Edge Case: Send Message</t>
+          <t>Boundary: Send Message</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -4996,30 +5878,29 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Verify sending message while receiver is typing</t>
+          <t>Verify sending text message with exactly 1 character</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1. Both users type simultaneously.
-2. Both send at the same time.</t>
+          <t>1. Send 'a'.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Both messages should appear in correct order. No message loss.</t>
+          <t>Single character message should send and display correctly.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>Low / Low</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MSG_120</t>
+          <t>MSG_126</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -5027,60 +5908,63 @@
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Verify sending message to a user who blocked you</t>
+          <t>Verify sending text at max character limit</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1. Send a message to a user who has blocked you.</t>
+          <t>1. Send a message at exactly the maximum character limit.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Message should fail or appear sent but not delivered. Appropriate handling per app policy.</t>
+          <t>Message should send successfully.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MSG_121</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n"/>
+          <t>MSG_128</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
       <c r="C4" s="2" t="n"/>
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Verify sending message immediately after joining a group</t>
+          <t>Verify sending media at minimum file size (1 byte)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>1. Join a new group.
-2. Immediately send a message.</t>
+          <t>1. Send a 1-byte file.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Message should send successfully. Should appear for all group members.</t>
+          <t>File should either send or be rejected as too small. No crash.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Medium / Medium</t>
+          <t>Low / Low</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>MSG_122</t>
+          <t>MSG_129</t>
         </is>
       </c>
       <c r="B5" s="2" t="n"/>
@@ -5088,41 +5972,39 @@
       <c r="D5" s="2" t="n"/>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Verify sending multiple media types in sequence</t>
+          <t>Verify sending media at exactly max file size</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>1. Send an image.
-2. Immediately send a video.
-3. Send a document.</t>
+          <t>1. Send a file at exactly the maximum allowed size.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>All three should upload and appear in correct order. No upload conflicts.</t>
+          <t>File should upload and send successfully.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>High / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>MSG_123</t>
+          <t>MSG_127</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -5130,77 +6012,52 @@
           <t>Negative</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Edge Case: Send Message</t>
-        </is>
-      </c>
+      <c r="C7" s="2" t="n"/>
       <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Verify sending message with zero-width characters</t>
+          <t>Verify sending text exceeding max character limit</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1. Send a message containing only zero-width unicode characters.</t>
+          <t>1. Try to send a message exceeding the max limit.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Message should be blocked or displayed as empty. No invisible messages.</t>
+          <t>Should be blocked at input or rejected by server with error.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Medium / High</t>
+          <t>Medium / Medium</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>MSG_124</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Verify sending corrupted media file</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>1. Rename a .txt file to .jpg.
-2. Try to send as image.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>App should detect invalid file and show error. Should not crash.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Medium / High</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
+      <c r="C8" s="4" t="n"/>
+      <c r="D8" s="4" t="n"/>
+      <c r="E8" s="4" t="n"/>
+      <c r="F8" s="4" t="n"/>
+      <c r="G8" s="4" t="n"/>
+      <c r="H8" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="007030A0"/>
+    <tabColor rgb="0000B0F0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5258,7 +6115,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MSG_125</t>
+          <t>MSG_130</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -5268,39 +6125,40 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Boundary: Send Message</t>
+          <t>Equivalence Partitioning: Message Destinations</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>User is logged in and chat is open</t>
+          <t>User is logged in</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Verify sending text message with exactly 1 character</t>
+          <t>Verify sending message in one-on-one chat</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>1. Send 'a'.</t>
+          <t>1. Open a one-on-one conversation.
+2. Send a text message.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Single character message should send and display correctly.</t>
+          <t>Message should deliver to the single recipient.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Low / Low</t>
+          <t>High / High</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>MSG_126</t>
+          <t>MSG_131</t>
         </is>
       </c>
       <c r="B3" s="2" t="n"/>
@@ -5308,254 +6166,6 @@
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Verify sending text at max character limit</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>1. Send a message at exactly the maximum character limit.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Message should send successfully.</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>MSG_128</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Verify sending media at minimum file size (1 byte)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>1. Send a 1-byte file.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>File should either send or be rejected as too small. No crash.</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Low / Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>MSG_129</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Verify sending media at exactly max file size</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>1. Send a file at exactly the maximum allowed size.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>File should upload and send successfully.</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>MSG_127</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>Negative</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Verify sending text exceeding max character limit</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>1. Try to send a message exceeding the max limit.</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Should be blocked at input or rejected by server with error.</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Medium / Medium</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="0000B0F0"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="45" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>TestCase_ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Sentiment</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Test Scenario</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Precondition</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Test Case</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Steps</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Results</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Priority / Severity</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>MSG_130</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Equivalence Partitioning: Message Destinations</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>User is logged in</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Verify sending message in one-on-one chat</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>1. Open a one-on-one conversation.
-2. Send a text message.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Message should deliver to the single recipient.</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>High / High</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>MSG_131</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
           <t>Verify sending message in small group (2-10 members)</t>
         </is>
       </c>
@@ -5923,6 +6533,16 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="4" t="n"/>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
+      <c r="E15" s="4" t="n"/>
+      <c r="F15" s="4" t="n"/>
+      <c r="G15" s="4" t="n"/>
+      <c r="H15" s="4" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>